<commit_message>
Fix Photo 5 captions (Pro), correct q230 text, remove claim phrases from 130 descriptions, add package size and weight
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HWYbtgoYaqPRgjtpLVjpZo
</commit_message>
<xml_diff>
--- a/Airpods pro_Pro2_406516.xlsx
+++ b/Airpods pro_Pro2_406516.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring desert climbing stamp trio design. Row of three retro travel-stamp illustrations with climbing gear, a starry desert night and a spiky desert tree. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring desert climbing stamp trio design. Row of three retro travel-stamp illustrations with climbing gear, a starry desert night and a spiky desert tree. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring park ranger stamp trio design. Row of three retro travel-stamp illustrations with a colourful hot spring, a ranger hat with binoculars and a bison. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring park ranger stamp trio design. Row of three retro travel-stamp illustrations with a colourful hot spring, a ranger hat with binoculars and a bison. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring peony and raspberry spray design. Watercolour-style botanical spray of a pink peony with raspberries and green leaves. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring peony and raspberry spray design. Watercolour-style botanical spray of a pink peony with raspberries and green leaves. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring gothic dark bloom flash design. Gothic tattoo-flash style row of dark roses, cameo, bow and crescent moon with a small ribbon banner. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring gothic dark bloom flash design. Gothic tattoo-flash style row of dark roses, cameo, bow and crescent moon with a small ribbon banner. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring gothic bat and roses design. Ornate gothic emblem with a crimson-winged bat, gold filigree, crescent moons and dark red roses. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring gothic bat and roses design. Ornate gothic emblem with a crimson-winged bat, gold filigree, crescent moons and dark red roses. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring cherries and blossoms design. Delicate watercolour-style spray of red cherries, pink blossoms and small blue flowers. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring cherries and blossoms design. Delicate watercolour-style spray of red cherries, pink blossoms and small blue flowers. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring walking pears badge design. Retro oval sticker-style badge with two smiling cartoon pears walking side by side and a playful fruit slogan. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring walking pears badge design. Retro oval sticker-style badge with two smiling cartoon pears walking side by side and a playful fruit slogan. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring forest camping stamp trio design. Row of three retro travel-stamp illustrations with a camping tent, a giant redwood and a granite mountain dome. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring forest camping stamp trio design. Row of three retro travel-stamp illustrations with a camping tent, a giant redwood and a granite mountain dome. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring lighthouse falcon stamp trio design. Row of three retro travel-stamp illustrations with a lighthouse on cliffs, a perched falcon and a coastal sunrise. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring lighthouse falcon stamp trio design. Row of three retro travel-stamp illustrations with a lighthouse on cliffs, a perched falcon and a coastal sunrise. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring blueberries and blue blossoms design. Delicate watercolour-style spray of blueberries with small blue flowers and green leaves. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring blueberries and blue blossoms design. Delicate watercolour-style spray of blueberries with small blue flowers and green leaves. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring orange popsicle sticker design. Retro sticker-style banner with an orange popsicle and an orange slice on a pink background with a fruity slogan. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring orange popsicle sticker design. Retro sticker-style banner with an orange popsicle and an orange slice on a pink background with a fruity slogan. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring running orange mascot design. Retro cartoon sticker of a cheerful running orange character with a bold citrus greeting. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring running orange mascot design. Retro cartoon sticker of a cheerful running orange character with a bold citrus greeting. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring reclining leopard wild luxe design. Vintage-style illustration of a reclining spotted leopard among tropical leaves with an elegant label. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring reclining leopard wild luxe design. Vintage-style illustration of a reclining spotted leopard among tropical leaves with an elegant label. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring mosaic cat with pineapples design. Whimsical folk-art mosaic cat in a red headscarf and boots surrounded by little pineapples. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring mosaic cat with pineapples design. Whimsical folk-art mosaic cat in a red headscarf and boots surrounded by little pineapples. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring tuxedo cat just coasting design. Cute cartoon sticker of a tuxedo cat riding an ocean wave with a laid-back slogan. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring tuxedo cat just coasting design. Cute cartoon sticker of a tuxedo cat riding an ocean wave with a laid-back slogan. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring swimming dachshund design. Cute cartoon dachshund stretched out swimming among little blue bubbles. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring swimming dachshund design. Cute cartoon dachshund stretched out swimming among little blue bubbles. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring sleepy bear hammock design. Cute camping sticker of a sleepy bear lounging in a hammock between pine trees with a punny slogan. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring sleepy bear hammock design. Cute camping sticker of a sleepy bear lounging in a hammock between pine trees with a punny slogan. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring dog riding rainbow fish design. Whimsical cartoon of a small corgi-style dog lounging on the back of a colourful fish. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring dog riding rainbow fish design. Whimsical cartoon of a small corgi-style dog lounging on the back of a colourful fish. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2077,17 +2077,17 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Black matte protective AirPods charging case cover with a black carabiner clip; the print is applied on the front of the cover. Print: Centred cartoon of a grinning scientist with spiky white hair, goggles on the forehead and a white lab coat, holding a bubbling green potion flask in one purple-gloved hand and a test tube in the other. Bold black outlines with white, purple, green and teal colours, printed directly on the black case.</t>
+          <t>Black matte protective AirPods charging case cover with a black carabiner clip; the print is applied on the front of the cover. Print: Centred cartoon of a grinning figure with spiky white and teal hair, a white outfit with green buttons and purple gloves, holding a bubbling green flask in one hand and a teal tool in the other. Bold black outlines with white, teal, green and purple colours, printed directly on the black case.</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring cartoon scientist with potions design. Fun cartoon scientist with spiky white hair and goggles holding bubbling green potions. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring spiky hair figure with green flask design. Smiling figure with spiky white and teal hair, a white outfit and purple gloves, holding a bubbling green flask in one hand and a teal tool in the other; white, teal, green and purple on black. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Black / Cartoon Scientist With Potions</t>
+          <t>Black / Spiky Hair Figure Green Flask</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring ready to learn backpack design. Cheerful back-to-school sticker art with a pink cartoon backpack and bubbly 'Ready to Learn!' lettering in yellow and pink. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring ready to learn backpack design. Cheerful back-to-school sticker art with a pink cartoon backpack and bubbly 'Ready to Learn!' lettering in yellow and pink. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring keep going smiling pencil design. Motivational school design with a smiling cartoon pencil, a pink A+ grade and bold 'Keep Going!' bubble lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring keep going smiling pencil design. Motivational school design with a smiling cartoon pencil, a pink A+ grade and bold 'Keep Going!' bubble lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring koi fish rising sun waves design. Japanese-style design of red and black koi fish circling a red sun above stylised ocean waves and pink cherry blossoms. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring koi fish rising sun waves design. Japanese-style design of red and black koi fish circling a red sun above stylised ocean waves and pink cherry blossoms. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring punk mode cassette design. Punk-rock banner with a hot-pink cassette tape, 'Punk Mode' lettering, checkered flags, safety pins and cyan lightning bolts. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring punk mode cassette design. Punk-rock banner with a hot-pink cassette tape, 'Punk Mode' lettering, checkered flags, safety pins and cyan lightning bolts. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring class vibes school collage design. Retro back-to-school sticker collage with a backpack, notebook, smiley face, daisy and rainbow plus 'Class Vibes' bubble lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring class vibes school collage design. Retro back-to-school sticker collage with a backpack, notebook, smiley face, daisy and rainbow plus 'Class Vibes' bubble lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring no rules rock hand design. Punk-rock banner with 'No Rules' lettering, a pink rock-on hand sign, checkered flags and cyan lightning bolts. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring no rules rock hand design. Punk-rock banner with 'No Rules' lettering, a pink rock-on hand sign, checkered flags and cyan lightning bolts. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring blue and pink butterflies design. Folk-art style blue and pink butterflies with green leafy sprigs and tiny flowers. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring blue and pink butterflies design. Folk-art style blue and pink butterflies with green leafy sprigs and tiny flowers. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring pizza thief cat design. Funny cartoon orange tabby cat snatching a slice of pizza with yellow 'Mine Now' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring pizza thief cat design. Funny cartoon orange tabby cat snatching a slice of pizza with yellow 'Mine Now' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring no risk no story lettering design. Bold retro hand-lettered quote 'No Risk No Story' in red and pink with lime-green sparkles. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring no risk no story lettering design. Bold retro hand-lettered quote 'No Risk No Story' in red and pink with lime-green sparkles. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring busy napping cat design. Cute cartoon black-and-white cat with a sleep mask napping on a keyboard, with 'Busy Napping' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring busy napping cat design. Cute cartoon black-and-white cat with a sleep mask napping on a keyboard, with 'Busy Napping' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring good vibes retro lettering design. Retro groovy 'Good Vibes' bubble lettering in pink and red with a wavy blue line and a little sun. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring good vibes retro lettering design. Retro groovy 'Good Vibes' bubble lettering in pink and red with a wavy blue line and a little sun. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring usa map lettering design. Patriotic blue United States map with stars and bold white 'USA' lettering with red accents. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring usa map lettering design. Patriotic blue United States map with stars and bold white 'USA' lettering with red accents. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring land of the free flag design. Patriotic waving stars-and-stripes flag with 'Land of the Free' white lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring land of the free flag design. Patriotic waving stars-and-stripes flag with 'Land of the Free' white lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring coastal road trip design. Coastal road-trip collage with a red suspension bridge, sailboat, sunset palms and a vintage red convertible with 'Coast' banner. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring coastal road trip design. Coastal road-trip collage with a red suspension bridge, sailboat, sunset palms and a vintage red convertible with 'Coast' banner. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring zero regrets snack cat design. Funny cartoon cat diving into a pink chip bag labelled 'Zero Regrets', with scattered yellow chips. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring zero regrets snack cat design. Funny cartoon cat diving into a pink chip bag labelled 'Zero Regrets', with scattered yellow chips. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring perfect fit box cat design. Cute cartoon black cat sitting in a pink box with a measuring tape and 'Perfect Fit' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring perfect fit box cat design. Cute cartoon black cat sitting in a pink box with a measuring tape and 'Perfect Fit' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring navy patterned sardines design. Mediterranean-style patterned sardine fish in cream and navy with little lemon wedges. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring navy patterned sardines design. Mediterranean-style patterned sardine fish in cream and navy with little lemon wedges. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring floral cowgirl bull skull design. Western folk-art bull skull wearing a pink cowboy hat, framed by horseshoes and colourful flowers. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring floral cowgirl bull skull design. Western folk-art bull skull wearing a pink cowboy hat, framed by horseshoes and colourful flowers. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring enchanted night halloween design. Cute Halloween banner with a little ghost, pumpkins, purple roses and bats with 'Enchanted Night' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring enchanted night halloween design. Cute Halloween banner with a little ghost, pumpkins, purple roses and bats with 'Enchanted Night' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring witchy mood pumpkins design. Spooky-cute Halloween design with a witch hand, skeleton hand, pumpkins and flowers framed by 'Witchy Mood' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring witchy mood pumpkins design. Spooky-cute Halloween design with a witch hand, skeleton hand, pumpkins and flowers framed by 'Witchy Mood' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring study break collage design. Retro study-themed sticker collage with books, calculator, smiley coffee cup and rainbow plus 'Study Break' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring study break collage design. Retro study-themed sticker collage with books, calculator, smiley coffee cup and rainbow plus 'Study Break' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring colourful daisy row design. Bright folk-style row of white, coral and pink daisies with green leaves. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring colourful daisy row design. Bright folk-style row of white, coral and pink daisies with green leaves. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring blueberry branch design. Cute illustrated blueberry branch with green leaves and a few pink berries. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring blueberry branch design. Cute illustrated blueberry branch with green leaves and a few pink berries. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring glam leopard on sofa design. Glamorous cartoon leopard in sunglasses lounging on a hot-pink sofa with a feather fan. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring glam leopard on sofa design. Glamorous cartoon leopard in sunglasses lounging on a hot-pink sofa with a feather fan. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring martini glass tiger design. Fun cartoon tiger in sunglasses lounging in a giant martini glass with a pink feather boa. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring martini glass tiger design. Fun cartoon tiger in sunglasses lounging in a giant martini glass with a pink feather boa. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring kitsune mask with fans design. Japanese-style white fox mask with folding fans, swirling clouds and cherry blossoms. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring kitsune mask with fans design. Japanese-style white fox mask with folding fans, swirling clouds and cherry blossoms. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring large pink butterfly design. Large decorative butterfly with cream and pink patterned wings. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring large pink butterfly design. Large decorative butterfly with cream and pink patterned wings. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring three coquette bows design. Coquette-style trio of blue, pink and green ribbon bows with little flowers. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring three coquette bows design. Coquette-style trio of blue, pink and green ribbon bows with little flowers. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring fishy business cat tin design. Cute cartoon black cat in a sardine tin with pink fish and 'Fishy Business' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring fishy business cat tin design. Cute cartoon black cat in a sardine tin with pink fish and 'Fishy Business' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring royal mess cat design. Funny cartoon black cat with a crown tangled in toilet paper, with 'Royal Mess' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring royal mess cat design. Funny cartoon black cat with a crown tangled in toilet paper, with 'Royal Mess' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring stretching leopard tropical design. Bright illustration of a stretching leopard among yellow starbursts, pink flowers and tropical leaves. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring stretching leopard tropical design. Bright illustration of a stretching leopard among yellow starbursts, pink flowers and tropical leaves. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring neon pink leopard head design. Realistic leopard head with neon pink star, lightning bolts and little stars. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring neon pink leopard head design. Realistic leopard head with neon pink star, lightning bolts and little stars. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring you got this smiling book design. Motivational 'You Got This!' bubble lettering above a smiling cartoon open book. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring you got this smiling book design. Motivational 'You Got This!' bubble lettering above a smiling cartoon open book. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring low poly green frog design. Geometric low-poly origami-style green frog. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring low poly green frog design. Geometric low-poly origami-style green frog. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring one eyed green monster design. Comic-style one-eyed green alien monster with sharp claws peeking out. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring one eyed green monster design. Comic-style one-eyed green alien monster with sharp claws peeking out. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring psychedelic peace smiley design. Retro psychedelic collage with a smiling sun, peace-sign hand, rainbows and flowers. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring psychedelic peace smiley design. Retro psychedelic collage with a smiling sun, peace-sign hand, rainbows and flowers. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring portal tabby cat design. Surreal tabby cat stepping through two rainbow portals. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring portal tabby cat design. Surreal tabby cat stepping through two rainbow portals. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring fluffy cat with burger design. Cute fluffy white cat lying on its back holding a cheeseburger. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring fluffy cat with burger design. Cute fluffy white cat lying on its back holding a cheeseburger. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring winging it hiking goose design. Funny cartoon hiking goose with a backpack and 'Winging It' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring winging it hiking goose design. Funny cartoon hiking goose with a backpack and 'Winging It' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring psychedelic mushrooms design. Trippy retro cluster of colourful polka-dot mushrooms under a crescent moon and stars. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring psychedelic mushrooms design. Trippy retro cluster of colourful polka-dot mushrooms under a crescent moon and stars. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring working my magic wizard design. Funny cartoon wizard typing on a retro computer with 'Working My Magic' lettering. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring working my magic wizard design. Funny cartoon wizard typing on a retro computer with 'Working My Magic' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring cat riding big fish design. Whimsical vintage-style illustration of a cat napping on top of a large colourful fish. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring cat riding big fish design. Whimsical vintage-style illustration of a cat napping on top of a large colourful fish. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring robot cowboy gunslinger design. Retro sci-fi robot cowboy gunslinger with orange hat and twin revolvers. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring robot cowboy gunslinger design. Retro sci-fi robot cowboy gunslinger with orange hat and twin revolvers. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring neon lucky cat torii design. Neon Japanese-style beckoning lucky cat with torii gate, fan, waves and cherry blossom. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring neon lucky cat torii design. Neon Japanese-style beckoning lucky cat with torii gate, fan, waves and cherry blossom. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring cartoon vampire count design. Comic-style vampire with fangs and a red high-collared cape reaching forward with clawed hands. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring cartoon vampire count design. Comic-style vampire with fangs and a red high-collared cape reaching forward with clawed hands. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring red white blue dots design. Abstract scattered red, white and navy confetti dots. Built as a black matte protective cover with a carabiner clip, precise cut-outs and full access to the charging port. Slim, lightweight protection against everyday scratches and bumps. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring red white blue dots design. Abstract scattered red, white and navy confetti dots. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Agent 1 batch US-AIRPODS-20261007-001: 130 listings, handoff JSONL, review XLSX, q246 renamed, validator decimal fix
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HWYbtgoYaqPRgjtpLVjpZo
</commit_message>
<xml_diff>
--- a/Airpods pro_Pro2_406516.xlsx
+++ b/Airpods pro_Pro2_406516.xlsx
@@ -2989,17 +2989,17 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Black matte protective AirPods charging case cover with a black carabiner clip; the print is applied on the front of the cover. Print: Centred cartoon of a black cat with big yellow eyes sitting in a pink box, wrapped by a lilac measuring tape, between the words 'PERFECT' in lilac and 'FIT' in yellow-green lettering, with a green crescent and sparkles. Sticker style, no background.</t>
+          <t>Black matte protective AirPods charging case cover with a black carabiner clip; the print is applied on the front of the cover. Print: Centred cartoon of a black cat with big yellow eyes sitting in a pink box, wrapped by a lilac measuring tape, between two words of lettering in lilac and yellow-green, with a green crescent and sparkles. Sticker style, no background.</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Decorative earbuds case cover featuring perfect fit box cat design. Cute cartoon black cat sitting in a pink box with a measuring tape and 'Perfect Fit' lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
+          <t>Decorative earbuds case cover featuring box cat lettering design. Cute cartoon black cat sitting in a pink box with a measuring tape and two words of lettering. Built as a black matte protective cover with a carabiner clip. Compatible with AirPods Pro / Pro 2.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Black / Perfect Fit Box Cat</t>
+          <t>Black / Box Cat Lettering</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">

</xml_diff>